<commit_message>
vp all labs upload
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="18">
   <si>
     <t xml:space="preserve">Предмет</t>
   </si>
@@ -40,7 +40,7 @@
 В ином случае нужно будет на сессии защищать работу на ноуте или удаленном подключении к своему компу домой   </t>
   </si>
   <si>
-    <t xml:space="preserve">Нет</t>
+    <t xml:space="preserve">Да</t>
   </si>
   <si>
     <t xml:space="preserve">Экономика</t>
@@ -50,16 +50,13 @@
 В контрольной делать только расчеты, анализ будем делать на сессии</t>
   </si>
   <si>
+    <t xml:space="preserve">Нет</t>
+  </si>
+  <si>
     <t xml:space="preserve">Архитектура ЭВМ</t>
   </si>
   <si>
-    <t xml:space="preserve">ЭИОС нет, группа в ТГ для вопросов.
-Материалы все скачаны на жд
-7 лаб + контрольная
-https://drive.google.com/drive/folders/1H6ScvnkuCvuDO-0YItXoDSzSuIaRKvZa?usp=drive_link (мой гугл диск)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Да</t>
+    <t xml:space="preserve">ЭИОС нет, группа в ТГ для вопросов. Материалы все скачаны на жд  7 лаб + контрольная</t>
   </si>
   <si>
     <t xml:space="preserve">Специальные главы математического анализа</t>
@@ -140,10 +137,9 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -537,7 +533,7 @@
       </c>
       <c r="L2" s="8" t="n">
         <f aca="false">(COUNTIF(C2:K2,"Да")/(COUNTIF(C2:K2,"Да")+COUNTIF(C2:K2,"Нет")))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="83.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -547,29 +543,15 @@
       <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>5</v>
-      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
       <c r="K3" s="7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L3" s="8" t="n">
         <f aca="false">(COUNTIF(C3:K3,"Да")/(COUNTIF(C3:K3,"Да")+COUNTIF(C3:K3,"Нет")))</f>
@@ -578,36 +560,36 @@
     </row>
     <row r="4" customFormat="false" ht="76.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>5</v>
-      </c>
       <c r="G4" s="7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I4" s="7"/>
       <c r="K4" s="7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L4" s="8" t="n">
         <f aca="false">(COUNTIF(C4:K4,"Да")/(COUNTIF(C4:K4,"Да")+COUNTIF(C4:K4,"Нет")))</f>
-        <v>0.285714285714286</v>
+        <v>0.428571428571429</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -617,29 +599,15 @@
       <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>5</v>
-      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
       <c r="K5" s="7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L5" s="8" t="n">
         <f aca="false">(COUNTIF(C5:K5,"Да")/(COUNTIF(C5:K5,"Да")+COUNTIF(C5:K5,"Нет")))</f>
@@ -654,17 +622,17 @@
         <v>14</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>5</v>
       </c>
       <c r="L6" s="8" t="n">
         <f aca="false">(COUNTIF(C6:K6,"Да")/(COUNTIF(C6:K6,"Да")+COUNTIF(C6:K6,"Нет")))</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -675,33 +643,33 @@
         <v>16</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>5</v>
       </c>
       <c r="J7" s="7"/>
       <c r="K7" s="7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L7" s="8" t="n">
         <f aca="false">(COUNTIF(C7:K7,"Да")/(COUNTIF(C7:K7,"Да")+COUNTIF(C7:K7,"Нет")))</f>
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -742,14 +710,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:H5 K2:K7 I3:I5 C6:D7 E7:J7 C8" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:H2 K2:K7 C3:I5 C6:D7 E7:J7 C8" type="list">
       <formula1>"Да,Нет"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" display="ЭИОС нет, группа в ТГ для вопросов.&#10;Материалы все скачаны на жд&#10;&#10;7 лаб + контрольная&#10;https://drive.google.com/drive/folders/1H6ScvnkuCvuDO-0YItXoDSzSuIaRKvZa?usp=drive_link (мой гугл диск)"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>